<commit_message>
actualice los archivos y ya funciona con pdfs
</commit_message>
<xml_diff>
--- a/documentos/EVALUACIONES MNM 2026.xlsx
+++ b/documentos/EVALUACIONES MNM 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29826"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29923"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Raúl\Dropbox (Personal)\2026\RESPALDO DE BASE DE DATOS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD9CFC01-7335-42B3-A99B-141667404703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF4CE410-6785-43C7-B549-86AAE1EF8F9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REPORTE" sheetId="5" r:id="rId1"/>
@@ -139,7 +139,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="115">
   <si>
     <t>NOMBRE DEL ALUMNO</t>
   </si>
@@ -544,6 +544,54 @@
   <si>
     <t>EQUIPO</t>
   </si>
+  <si>
+    <t>Eduardo Luis Diaz Olivo</t>
+  </si>
+  <si>
+    <t>Laura Ruiz Palomo</t>
+  </si>
+  <si>
+    <t>Miguel Castro Montes</t>
+  </si>
+  <si>
+    <t>Dario Restrepo Rojas</t>
+  </si>
+  <si>
+    <t>Saray Bastidas Pelaez</t>
+  </si>
+  <si>
+    <t>Santiago Peñates Ramos</t>
+  </si>
+  <si>
+    <t>Joel Jaraba Rosario</t>
+  </si>
+  <si>
+    <t>Angie Tatiana Patiño Segura</t>
+  </si>
+  <si>
+    <t>Evangely Bravo Padilla</t>
+  </si>
+  <si>
+    <t>Valeria Martinez Valero</t>
+  </si>
+  <si>
+    <t>Maria Carolina Tannus</t>
+  </si>
+  <si>
+    <t>Maria Fernanda Cogollo Cogollo</t>
+  </si>
+  <si>
+    <t>Elias Vergara Villalba</t>
+  </si>
+  <si>
+    <t>Ever Junior Polo Lozano</t>
+  </si>
+  <si>
+    <t>Sara Lucia Movilla Villalba</t>
+  </si>
+  <si>
+    <t>Valeria Guerra Machado</t>
+  </si>
 </sst>
 </file>
 
@@ -675,7 +723,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -792,11 +840,640 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="76">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor theme="0" tint="-0.14999847407452621"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="19" formatCode="d/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="165" formatCode="00"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1425,32 +2102,6 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor theme="0" tint="-0.14999847407452621"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
       <fill>
         <patternFill patternType="none">
           <fgColor theme="0" tint="-0.14999847407452621"/>
@@ -1816,425 +2467,6 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="19" formatCode="d/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="00"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
         <family val="2"/>
@@ -2497,142 +2729,6 @@
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -2883,7 +2979,7 @@
                   <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3086,7 +3182,7 @@
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3289,7 +3385,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -3692,7 +3788,7 @@
                         <c:v>35</c:v>
                       </c:pt>
                       <c:pt idx="2">
-                        <c:v>0</c:v>
+                        <c:v>34</c:v>
                       </c:pt>
                       <c:pt idx="3">
                         <c:v>0</c:v>
@@ -3860,7 +3956,7 @@
                         <c:v>1</c:v>
                       </c:pt>
                       <c:pt idx="2">
-                        <c:v>0</c:v>
+                        <c:v>4</c:v>
                       </c:pt>
                       <c:pt idx="3">
                         <c:v>0</c:v>
@@ -4639,7 +4735,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -5185,7 +5281,7 @@
                         <c:v>35</c:v>
                       </c:pt>
                       <c:pt idx="2">
-                        <c:v>0</c:v>
+                        <c:v>34</c:v>
                       </c:pt>
                       <c:pt idx="3">
                         <c:v>0</c:v>
@@ -5353,7 +5449,7 @@
                         <c:v>13</c:v>
                       </c:pt>
                       <c:pt idx="2">
-                        <c:v>0</c:v>
+                        <c:v>21</c:v>
                       </c:pt>
                       <c:pt idx="3">
                         <c:v>0</c:v>
@@ -5526,7 +5622,7 @@
                         <c:v>7</c:v>
                       </c:pt>
                       <c:pt idx="2">
-                        <c:v>0</c:v>
+                        <c:v>12</c:v>
                       </c:pt>
                       <c:pt idx="3">
                         <c:v>0</c:v>
@@ -5699,7 +5795,7 @@
                         <c:v>1</c:v>
                       </c:pt>
                       <c:pt idx="2">
-                        <c:v>0</c:v>
+                        <c:v>1</c:v>
                       </c:pt>
                       <c:pt idx="3">
                         <c:v>0</c:v>
@@ -6374,7 +6470,7 @@
                   <c:v>35</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -6560,7 +6656,7 @@
                         <c:v>13</c:v>
                       </c:pt>
                       <c:pt idx="2">
-                        <c:v>0</c:v>
+                        <c:v>21</c:v>
                       </c:pt>
                       <c:pt idx="3">
                         <c:v>0</c:v>
@@ -6733,7 +6829,7 @@
                         <c:v>1</c:v>
                       </c:pt>
                       <c:pt idx="2">
-                        <c:v>0</c:v>
+                        <c:v>4</c:v>
                       </c:pt>
                       <c:pt idx="3">
                         <c:v>0</c:v>
@@ -6906,7 +7002,7 @@
                         <c:v>7</c:v>
                       </c:pt>
                       <c:pt idx="2">
-                        <c:v>0</c:v>
+                        <c:v>12</c:v>
                       </c:pt>
                       <c:pt idx="3">
                         <c:v>0</c:v>
@@ -7252,7 +7348,7 @@
                         <c:v>1</c:v>
                       </c:pt>
                       <c:pt idx="2">
-                        <c:v>0</c:v>
+                        <c:v>1</c:v>
                       </c:pt>
                       <c:pt idx="3">
                         <c:v>0</c:v>
@@ -11923,7 +12019,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{DB9236B4-6758-46F5-ACE3-4324EBF03AFC}" name="Tabla11" displayName="Tabla11" ref="A1:I13" totalsRowShown="0" headerRowDxfId="69" dataDxfId="68">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{DB9236B4-6758-46F5-ACE3-4324EBF03AFC}" name="Tabla11" displayName="Tabla11" ref="A1:I13" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
   <autoFilter ref="A1:I13" xr:uid="{DB9236B4-6758-46F5-ACE3-4324EBF03AFC}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -11936,29 +12032,29 @@
     <filterColumn colId="8" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{E45CE681-0F10-4F5F-ABE9-36AD6411F2F4}" name="MESES" dataDxfId="67"/>
-    <tableColumn id="2" xr3:uid="{C45C8DBF-C350-4EAC-B340-B1433B532DF4}" name="T. ALUMNOS" dataDxfId="66">
+    <tableColumn id="1" xr3:uid="{E45CE681-0F10-4F5F-ABE9-36AD6411F2F4}" name="MESES" dataDxfId="73"/>
+    <tableColumn id="2" xr3:uid="{C45C8DBF-C350-4EAC-B340-B1433B532DF4}" name="T. ALUMNOS" dataDxfId="72">
       <calculatedColumnFormula>SUM(Tabla11[[#This Row],[TOTAL N1]],Tabla11[[#This Row],[TOTAL N2]],Tabla11[[#This Row],[TOTAL N3]],Tabla11[[#This Row],[T. EQUIPO]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{544D14A8-0150-477C-91EB-9C6A53287C61}" name="TOTAL N1" dataDxfId="65">
+    <tableColumn id="3" xr3:uid="{544D14A8-0150-477C-91EB-9C6A53287C61}" name="TOTAL N1" dataDxfId="71">
       <calculatedColumnFormula>COUNTIF('NIVEL 1'!$B:$B,REPORTE!A2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{B844FCB1-5911-4097-AC96-E45A77F4EADB}" name="CAMBIO N2" dataDxfId="64">
+    <tableColumn id="4" xr3:uid="{B844FCB1-5911-4097-AC96-E45A77F4EADB}" name="CAMBIO N2" dataDxfId="70">
       <calculatedColumnFormula>COUNTIFS('NIVEL 1'!$B:$B,Tabla11[[#This Row],[MESES]],'NIVEL 1'!$N:$N,"CAMBIA A NIVEL 2")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{09584C72-C135-48E6-BBF7-7505B75ADFE1}" name="TOTAL N2" dataDxfId="63">
+    <tableColumn id="6" xr3:uid="{09584C72-C135-48E6-BBF7-7505B75ADFE1}" name="TOTAL N2" dataDxfId="69">
       <calculatedColumnFormula>COUNTIF('NIVEL 2'!$B:$B,REPORTE!A2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{050D800C-3210-4B53-B962-4423AD8D7D44}" name="CAMBIO N3" dataDxfId="62">
+    <tableColumn id="7" xr3:uid="{050D800C-3210-4B53-B962-4423AD8D7D44}" name="CAMBIO N3" dataDxfId="68">
       <calculatedColumnFormula>COUNTIFS('NIVEL 2'!$B:$B,Tabla11[[#This Row],[MESES]],'NIVEL 2'!$N:$N,"CAMBIA A NIVEL 3")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{533A7FB5-2283-4C4B-B4C5-7CB89D8F9805}" name="TOTAL N3" dataDxfId="61">
+    <tableColumn id="9" xr3:uid="{533A7FB5-2283-4C4B-B4C5-7CB89D8F9805}" name="TOTAL N3" dataDxfId="67">
       <calculatedColumnFormula>COUNTIF('NIVEL 3'!$B:$B,REPORTE!A2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{A1B4EC19-A475-44A6-8767-A1367A64797F}" name="A EQUIPO" dataDxfId="60">
+    <tableColumn id="10" xr3:uid="{A1B4EC19-A475-44A6-8767-A1367A64797F}" name="A EQUIPO" dataDxfId="66">
       <calculatedColumnFormula>COUNTIFS('NIVEL 3'!$B:$B,Tabla11[[#This Row],[MESES]],'NIVEL 3'!$N:$N,"CAMBIA A EQUIPO")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{BB0919BB-10F2-4412-9120-0EF7216850C1}" name="T. EQUIPO" dataDxfId="59">
+    <tableColumn id="12" xr3:uid="{BB0919BB-10F2-4412-9120-0EF7216850C1}" name="T. EQUIPO" dataDxfId="65">
       <calculatedColumnFormula>COUNTIF(EQUIPO!$B:$B,REPORTE!A2)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -11967,37 +12063,37 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{AE1B38D2-F5E0-437E-A0C7-D4FAEDCDAD9F}" name="NIVEL_1" displayName="NIVEL_1" ref="A2:O25" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57" tableBorderDxfId="56">
-  <autoFilter ref="A2:O25" xr:uid="{AE1B38D2-F5E0-437E-A0C7-D4FAEDCDAD9F}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:O25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{AE1B38D2-F5E0-437E-A0C7-D4FAEDCDAD9F}" name="NIVEL_1" displayName="NIVEL_1" ref="A2:O46" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17" tableBorderDxfId="16">
+  <autoFilter ref="A2:O46" xr:uid="{AE1B38D2-F5E0-437E-A0C7-D4FAEDCDAD9F}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:O46">
     <sortCondition ref="D3:D25"/>
     <sortCondition ref="A3:A25"/>
     <sortCondition ref="F3:F25"/>
   </sortState>
   <tableColumns count="15">
-    <tableColumn id="15" xr3:uid="{06087576-FB0C-44ED-9CDF-C51BACC66F7B}" name="#" dataDxfId="55">
+    <tableColumn id="15" xr3:uid="{06087576-FB0C-44ED-9CDF-C51BACC66F7B}" name="#" dataDxfId="15">
       <calculatedColumnFormula>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{8EF9B412-985A-48AA-9792-B95947050FCB}" name="NIVEL" dataDxfId="54">
+    <tableColumn id="1" xr3:uid="{8EF9B412-985A-48AA-9792-B95947050FCB}" name="NIVEL" dataDxfId="14">
       <calculatedColumnFormula>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{2E9F9510-35A9-488E-B1DE-D74FC37EE91B}" name="MES" dataDxfId="53">
+    <tableColumn id="2" xr3:uid="{2E9F9510-35A9-488E-B1DE-D74FC37EE91B}" name="MES" dataDxfId="13">
       <calculatedColumnFormula>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{9F822B2A-0A90-4E18-A961-AC7ADB5E33D7}" name="Fecha de Evaluación" dataDxfId="52"/>
-    <tableColumn id="4" xr3:uid="{F1A37849-EC75-4EFB-8761-8B4816148787}" name="NOMBRE DEL ALUMNO" dataDxfId="51"/>
-    <tableColumn id="5" xr3:uid="{75F8F1A3-4C2C-48D8-BDA8-8EDA5D423C89}" name="DOCUMENTO" dataDxfId="50"/>
-    <tableColumn id="6" xr3:uid="{C323AA94-0265-4893-9265-35B1038BBE77}" name="AMBIENTACION" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{508CEACB-AA59-433A-AFBE-23B4CF5354AF}" name="FLOTACION DEFENSIVA" dataDxfId="48"/>
-    <tableColumn id="8" xr3:uid="{596F9D83-7601-4A50-9A71-07FA546F1FDC}" name="PATADA CROL" dataDxfId="47"/>
-    <tableColumn id="9" xr3:uid="{1386C268-2BDD-48F8-9EC7-CB447E9A76B9}" name="PADATA ESPALDA" dataDxfId="46"/>
-    <tableColumn id="10" xr3:uid="{B76B36D4-2E2E-4645-8403-BA569067D6EB}" name="ENS. CROL" dataDxfId="45"/>
-    <tableColumn id="11" xr3:uid="{A284663E-58C2-40EC-80B3-D1F680E97AF3}" name="ENS ESPALDA" dataDxfId="44"/>
-    <tableColumn id="12" xr3:uid="{EA24CD10-C3F1-45CB-A915-9CB5EA29D8A1}" name="SALTO" dataDxfId="43"/>
-    <tableColumn id="13" xr3:uid="{95D67B47-0B42-429F-9EC3-5161FF1E86D0}" name="Pase de Nivel 4,7 ptos" dataDxfId="42">
+    <tableColumn id="3" xr3:uid="{9F822B2A-0A90-4E18-A961-AC7ADB5E33D7}" name="Fecha de Evaluación" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{F1A37849-EC75-4EFB-8761-8B4816148787}" name="NOMBRE DEL ALUMNO" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{75F8F1A3-4C2C-48D8-BDA8-8EDA5D423C89}" name="DOCUMENTO" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{C323AA94-0265-4893-9265-35B1038BBE77}" name="AMBIENTACION" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{508CEACB-AA59-433A-AFBE-23B4CF5354AF}" name="FLOTACION DEFENSIVA" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{596F9D83-7601-4A50-9A71-07FA546F1FDC}" name="PATADA CROL" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{1386C268-2BDD-48F8-9EC7-CB447E9A76B9}" name="PADATA ESPALDA" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{B76B36D4-2E2E-4645-8403-BA569067D6EB}" name="ENS. CROL" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{A284663E-58C2-40EC-80B3-D1F680E97AF3}" name="ENS ESPALDA" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{EA24CD10-C3F1-45CB-A915-9CB5EA29D8A1}" name="SALTO" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{95D67B47-0B42-429F-9EC3-5161FF1E86D0}" name="Pase de Nivel 4,7 ptos" dataDxfId="1">
       <calculatedColumnFormula>IFERROR(AVERAGE('NIVEL 1'!G3:M3),"-")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{20659D21-4226-4F1C-9913-990D646166B3}" name="Cambio de Nivel" dataDxfId="41">
+    <tableColumn id="14" xr3:uid="{20659D21-4226-4F1C-9913-990D646166B3}" name="Cambio de Nivel" dataDxfId="2">
       <calculatedColumnFormula array="1">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -12006,36 +12102,36 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{D3B83B8F-7030-4C6B-865D-1CEF5FF0A135}" name="NIVEL_2" displayName="NIVEL_2" ref="A2:O11" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
-  <autoFilter ref="A2:O11" xr:uid="{D3B83B8F-7030-4C6B-865D-1CEF5FF0A135}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:O11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{D3B83B8F-7030-4C6B-865D-1CEF5FF0A135}" name="NIVEL_2" displayName="NIVEL_2" ref="A2:O23" totalsRowShown="0" headerRowDxfId="64" dataDxfId="63">
+  <autoFilter ref="A2:O23" xr:uid="{D3B83B8F-7030-4C6B-865D-1CEF5FF0A135}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:O23">
     <sortCondition ref="A3:A4"/>
     <sortCondition ref="F3:F4"/>
   </sortState>
   <tableColumns count="15">
-    <tableColumn id="15" xr3:uid="{09B76DB3-82BE-4C0B-B453-BF194A257258}" name="#" dataDxfId="38">
+    <tableColumn id="15" xr3:uid="{09B76DB3-82BE-4C0B-B453-BF194A257258}" name="#" dataDxfId="62">
       <calculatedColumnFormula>MONTH(NIVEL_2[[#This Row],[Fecha de Evaluación]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{A30C7826-C605-4AD6-9BD1-976B3108B364}" name="NIVEL" dataDxfId="37">
+    <tableColumn id="1" xr3:uid="{A30C7826-C605-4AD6-9BD1-976B3108B364}" name="NIVEL" dataDxfId="61">
       <calculatedColumnFormula>IF(NIVEL_2[[#This Row],['#]]&gt;0,"NIVEL 2","")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{278C7F91-1379-491F-9B18-95B5FB0F5B4C}" name="MES" dataDxfId="36">
+    <tableColumn id="2" xr3:uid="{278C7F91-1379-491F-9B18-95B5FB0F5B4C}" name="MES" dataDxfId="60">
       <calculatedColumnFormula>TEXT(NIVEL_2[[#This Row],[Fecha de Evaluación]],"MMMM")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{61734E93-B6EC-4BCE-81B8-694554146D51}" name="Fecha de Evaluación" dataDxfId="35"/>
-    <tableColumn id="4" xr3:uid="{52287499-B96A-4EC4-9C46-4A9605C862D7}" name="NOMBRE DEL ALUMNO" dataDxfId="34"/>
-    <tableColumn id="5" xr3:uid="{0ECA98BC-FB01-4F67-8A05-CB651A1C8B21}" name="DOCUMENTO" dataDxfId="33"/>
-    <tableColumn id="6" xr3:uid="{4E959843-5A00-4667-9538-531D9390ABDE}" name="TECN ESTILO CROL" dataDxfId="32"/>
-    <tableColumn id="7" xr3:uid="{D6B9A5DE-DA9B-48F2-BC77-F1A1DF233559}" name="TECN ESTILO ESPAL" dataDxfId="31"/>
-    <tableColumn id="8" xr3:uid="{3674AFCF-043A-4668-A622-83DFE8ED6907}" name="ENSE EST PECHO" dataDxfId="30"/>
-    <tableColumn id="9" xr3:uid="{4E82D7B2-52CF-420D-97A4-0A59EFC666C9}" name="ENSE EST MARIPOSA" dataDxfId="29"/>
-    <tableColumn id="10" xr3:uid="{BF17361D-FC57-499E-9503-C2F33EB21C88}" name="INI SALIDA OLIMPICA" dataDxfId="28"/>
-    <tableColumn id="11" xr3:uid="{8B1BEFD7-6FF5-425A-89DA-581562D0A38F}" name="50 m LIBRE" dataDxfId="27"/>
-    <tableColumn id="12" xr3:uid="{991D9CFF-9F59-44B7-AA62-F62FE91F51E4}" name="INI VUELTA OLIMPICA" dataDxfId="26"/>
-    <tableColumn id="13" xr3:uid="{1083E4EB-1DAF-41A3-B727-7BF532F1CB2C}" name="Pase de Nivel 4,7 ptos" dataDxfId="25">
+    <tableColumn id="3" xr3:uid="{61734E93-B6EC-4BCE-81B8-694554146D51}" name="Fecha de Evaluación" dataDxfId="59"/>
+    <tableColumn id="4" xr3:uid="{52287499-B96A-4EC4-9C46-4A9605C862D7}" name="NOMBRE DEL ALUMNO" dataDxfId="58"/>
+    <tableColumn id="5" xr3:uid="{0ECA98BC-FB01-4F67-8A05-CB651A1C8B21}" name="DOCUMENTO" dataDxfId="57"/>
+    <tableColumn id="6" xr3:uid="{4E959843-5A00-4667-9538-531D9390ABDE}" name="TECN ESTILO CROL" dataDxfId="56"/>
+    <tableColumn id="7" xr3:uid="{D6B9A5DE-DA9B-48F2-BC77-F1A1DF233559}" name="TECN ESTILO ESPAL" dataDxfId="55"/>
+    <tableColumn id="8" xr3:uid="{3674AFCF-043A-4668-A622-83DFE8ED6907}" name="ENSE EST PECHO" dataDxfId="54"/>
+    <tableColumn id="9" xr3:uid="{4E82D7B2-52CF-420D-97A4-0A59EFC666C9}" name="ENSE EST MARIPOSA" dataDxfId="53"/>
+    <tableColumn id="10" xr3:uid="{BF17361D-FC57-499E-9503-C2F33EB21C88}" name="INI SALIDA OLIMPICA" dataDxfId="52"/>
+    <tableColumn id="11" xr3:uid="{8B1BEFD7-6FF5-425A-89DA-581562D0A38F}" name="50 m LIBRE" dataDxfId="51"/>
+    <tableColumn id="12" xr3:uid="{991D9CFF-9F59-44B7-AA62-F62FE91F51E4}" name="INI VUELTA OLIMPICA" dataDxfId="50"/>
+    <tableColumn id="13" xr3:uid="{1083E4EB-1DAF-41A3-B727-7BF532F1CB2C}" name="Pase de Nivel 4,7 ptos" dataDxfId="0">
       <calculatedColumnFormula>IFERROR(AVERAGE('NIVEL 2'!G3:M3),"-")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{EA8CA3F6-4262-42A0-A47A-543052CC352E}" name="Cambio de Nivel" dataDxfId="24">
+    <tableColumn id="14" xr3:uid="{EA8CA3F6-4262-42A0-A47A-543052CC352E}" name="Cambio de Nivel" dataDxfId="49">
       <calculatedColumnFormula array="1">_xlfn.IFS(NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 3",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -12044,42 +12140,42 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{1228A722-3B02-41C4-936F-4D7749F95EAB}" name="NIVEL_3" displayName="NIVEL_3" ref="A2:U5" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22" tableBorderDxfId="21">
-  <autoFilter ref="A2:U5" xr:uid="{1228A722-3B02-41C4-936F-4D7749F95EAB}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{1228A722-3B02-41C4-936F-4D7749F95EAB}" name="NIVEL_3" displayName="NIVEL_3" ref="A2:U6" totalsRowShown="0" headerRowDxfId="48" dataDxfId="47" tableBorderDxfId="46">
+  <autoFilter ref="A2:U6" xr:uid="{1228A722-3B02-41C4-936F-4D7749F95EAB}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:U4">
     <sortCondition ref="A3"/>
     <sortCondition ref="F3"/>
   </sortState>
   <tableColumns count="21">
-    <tableColumn id="20" xr3:uid="{323FD556-7D50-469A-834D-326AE7F31F42}" name="#" dataDxfId="20">
+    <tableColumn id="20" xr3:uid="{323FD556-7D50-469A-834D-326AE7F31F42}" name="#" dataDxfId="45">
       <calculatedColumnFormula>MONTH(NIVEL_3[[#This Row],[Fecha de Evaluación]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{10AF1518-13B3-40F9-A98E-94CD6E53DC3C}" name="NIVEL" dataDxfId="19">
+    <tableColumn id="21" xr3:uid="{10AF1518-13B3-40F9-A98E-94CD6E53DC3C}" name="NIVEL" dataDxfId="44">
       <calculatedColumnFormula>IF(NIVEL_3[[#This Row],['#]]&gt;0,"NIVEL 3","")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{EB57D90D-D066-4E6D-A973-52FAC5B51F0B}" name="MES" dataDxfId="18">
+    <tableColumn id="1" xr3:uid="{EB57D90D-D066-4E6D-A973-52FAC5B51F0B}" name="MES" dataDxfId="43">
       <calculatedColumnFormula>TEXT(NIVEL_3[[#This Row],[Fecha de Evaluación]],"MMMM")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0FF92161-361C-4203-A4D2-423DC120EB57}" name="Fecha de Evaluación" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{717B9D19-3A86-46A2-91B1-EC86BF2E533D}" name="NOMBRE DEL ALUMNO" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{C69B0C8E-7042-4239-BC38-5DE04F3B8AED}" name="DOCUMENTO" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{1EE2B091-87B8-431E-9319-6E87870DA8A7}" name="100m CROL" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{149128A8-27D9-491E-BD3D-385F53877A11}" name="VUELTA OLIMP. CROL" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{124D09B0-F954-4F41-A77B-869A1BDB006E}" name="LLEGADA CROL" dataDxfId="12"/>
-    <tableColumn id="8" xr3:uid="{350D03DD-5253-4CC2-BFB2-33A4611914A5}" name="SALIDA OLIMP. ESPALDA" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{06F7D230-4D74-4E3E-8042-C13E6EA69D7C}" name="100m ESPALDA" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{C7656A52-730D-4608-BED4-BE3F03A2F535}" name="VUELTA OLIMP. ESPALDA" dataDxfId="9"/>
-    <tableColumn id="11" xr3:uid="{826AA493-8CDE-43B4-9D76-F71252CD2636}" name="LLEGADA ESPALDA" dataDxfId="8"/>
-    <tableColumn id="12" xr3:uid="{EA88C99C-8AE3-41D5-88C9-4D1A205AE057}" name="SALIDA OLIMP. MARIPOSA" dataDxfId="7"/>
-    <tableColumn id="13" xr3:uid="{6446B914-DD25-438C-985E-231095C15D34}" name="25m MARIPOSA" dataDxfId="6"/>
-    <tableColumn id="14" xr3:uid="{ADF9866C-0662-48A4-BD02-64795FE4507E}" name="LLEGADA MARIPOSA" dataDxfId="5"/>
-    <tableColumn id="15" xr3:uid="{B9BF3AB6-845A-4D24-8DE1-E6713B1B6A8E}" name="SALIDA OLIMP. PECHO" dataDxfId="4"/>
-    <tableColumn id="16" xr3:uid="{66B4F0A1-9475-49BD-BDF4-157D5AF07759}" name="25m PECHO" dataDxfId="3"/>
-    <tableColumn id="17" xr3:uid="{C4433153-B84C-45D5-9DAA-18C80B367D88}" name="LLEGADA PECHO" dataDxfId="2"/>
-    <tableColumn id="18" xr3:uid="{3A6F3CA6-C52F-40C3-9659-D551D3CB8905}" name="Pase de Nivel 4,9 ptos" dataDxfId="1">
+    <tableColumn id="2" xr3:uid="{0FF92161-361C-4203-A4D2-423DC120EB57}" name="Fecha de Evaluación" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{717B9D19-3A86-46A2-91B1-EC86BF2E533D}" name="NOMBRE DEL ALUMNO" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{C69B0C8E-7042-4239-BC38-5DE04F3B8AED}" name="DOCUMENTO" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{1EE2B091-87B8-431E-9319-6E87870DA8A7}" name="100m CROL" dataDxfId="39"/>
+    <tableColumn id="6" xr3:uid="{149128A8-27D9-491E-BD3D-385F53877A11}" name="VUELTA OLIMP. CROL" dataDxfId="38"/>
+    <tableColumn id="7" xr3:uid="{124D09B0-F954-4F41-A77B-869A1BDB006E}" name="LLEGADA CROL" dataDxfId="37"/>
+    <tableColumn id="8" xr3:uid="{350D03DD-5253-4CC2-BFB2-33A4611914A5}" name="SALIDA OLIMP. ESPALDA" dataDxfId="36"/>
+    <tableColumn id="9" xr3:uid="{06F7D230-4D74-4E3E-8042-C13E6EA69D7C}" name="100m ESPALDA" dataDxfId="35"/>
+    <tableColumn id="10" xr3:uid="{C7656A52-730D-4608-BED4-BE3F03A2F535}" name="VUELTA OLIMP. ESPALDA" dataDxfId="34"/>
+    <tableColumn id="11" xr3:uid="{826AA493-8CDE-43B4-9D76-F71252CD2636}" name="LLEGADA ESPALDA" dataDxfId="33"/>
+    <tableColumn id="12" xr3:uid="{EA88C99C-8AE3-41D5-88C9-4D1A205AE057}" name="SALIDA OLIMP. MARIPOSA" dataDxfId="32"/>
+    <tableColumn id="13" xr3:uid="{6446B914-DD25-438C-985E-231095C15D34}" name="25m MARIPOSA" dataDxfId="31"/>
+    <tableColumn id="14" xr3:uid="{ADF9866C-0662-48A4-BD02-64795FE4507E}" name="LLEGADA MARIPOSA" dataDxfId="30"/>
+    <tableColumn id="15" xr3:uid="{B9BF3AB6-845A-4D24-8DE1-E6713B1B6A8E}" name="SALIDA OLIMP. PECHO" dataDxfId="29"/>
+    <tableColumn id="16" xr3:uid="{66B4F0A1-9475-49BD-BDF4-157D5AF07759}" name="25m PECHO" dataDxfId="28"/>
+    <tableColumn id="17" xr3:uid="{C4433153-B84C-45D5-9DAA-18C80B367D88}" name="LLEGADA PECHO" dataDxfId="27"/>
+    <tableColumn id="18" xr3:uid="{3A6F3CA6-C52F-40C3-9659-D551D3CB8905}" name="Pase de Nivel 4,9 ptos" dataDxfId="26">
       <calculatedColumnFormula>IFERROR(AVERAGE(G3:S3),"-")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{A6317C45-4DC3-4C83-B4AE-F03D89924519}" name="Cambio de Nivel" dataDxfId="0">
+    <tableColumn id="19" xr3:uid="{A6317C45-4DC3-4C83-B4AE-F03D89924519}" name="Cambio de Nivel" dataDxfId="25">
       <calculatedColumnFormula array="1">_xlfn.IFS(NIVEL_3[[#This Row],[Pase de Nivel 4,9 ptos]]="-","-",NIVEL_3[[#This Row],[Pase de Nivel 4,9 ptos]]&gt;=4.9,"CAMBIA A EQUIPO",NIVEL_3[[#This Row],[Pase de Nivel 4,9 ptos]]&lt;=4.9,"-")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -12088,17 +12184,17 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{C5681B1A-EC8A-41B9-A9DC-57C6B186CE75}" name="NIVEL_213" displayName="NIVEL_213" ref="A2:D138" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{C5681B1A-EC8A-41B9-A9DC-57C6B186CE75}" name="NIVEL_213" displayName="NIVEL_213" ref="A2:D138" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="A2:D138" xr:uid="{C5681B1A-EC8A-41B9-A9DC-57C6B186CE75}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:D33">
     <sortCondition ref="A3"/>
     <sortCondition ref="D3"/>
   </sortState>
   <tableColumns count="4">
-    <tableColumn id="5" xr3:uid="{6BE10E98-8110-4B32-B324-956C2A939720}" name="N°" dataDxfId="73"/>
-    <tableColumn id="1" xr3:uid="{47EC1D0D-C132-491F-995F-583089EB3DC6}" name="NIVEL" dataDxfId="72"/>
-    <tableColumn id="2" xr3:uid="{E3EBB2A9-A349-4F03-8A3C-7C71DFE91475}" name="MES" dataDxfId="71"/>
-    <tableColumn id="4" xr3:uid="{15956556-3BA8-42CE-A623-63D4505D4189}" name="NOMBRE DEL ALUMNO" dataDxfId="70"/>
+    <tableColumn id="5" xr3:uid="{6BE10E98-8110-4B32-B324-956C2A939720}" name="N°" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{47EC1D0D-C132-491F-995F-583089EB3DC6}" name="NIVEL" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{E3EBB2A9-A349-4F03-8A3C-7C71DFE91475}" name="MES" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{15956556-3BA8-42CE-A623-63D4505D4189}" name="NOMBRE DEL ALUMNO" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -12485,19 +12581,19 @@
       </c>
       <c r="B4" s="17">
         <f>SUM(Tabla11[[#This Row],[TOTAL N1]],Tabla11[[#This Row],[TOTAL N2]],Tabla11[[#This Row],[TOTAL N3]],Tabla11[[#This Row],[T. EQUIPO]])</f>
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="C4" s="17">
         <f>COUNTIF('NIVEL 1'!$C:$C,REPORTE!A4)</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="D4" s="17">
         <f>COUNTIFS('NIVEL 1'!$C:$C,Tabla11[[#This Row],[MESES]],'NIVEL 1'!$O:$O,"CAMBIA A NIVEL 2")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E4" s="17">
         <f>COUNTIF('NIVEL 2'!$C:$C,REPORTE!A4)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F4" s="17">
         <f>COUNTIFS('NIVEL 2'!$C:$C,Tabla11[[#This Row],[MESES]],'NIVEL 2'!$O:$O,"CAMBIA A NIVEL 3")</f>
@@ -12505,7 +12601,7 @@
       </c>
       <c r="G4" s="17">
         <f>COUNTIF('NIVEL 3'!$C:$C,REPORTE!A4)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="17">
         <f>COUNTIFS('NIVEL 3'!$C:$C,Tabla11[[#This Row],[MESES]],'NIVEL 3'!$U:$U,"CAMBIA A EQUIPO")</f>
@@ -12867,7 +12963,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O25"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.33203125" customWidth="1"/>
@@ -14143,6 +14239,1098 @@
       </c>
       <c r="O25" s="18" t="str" cm="1">
         <f t="array" ref="O25">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A26" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B26" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C26" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D26" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E26" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="F26" s="44">
+        <v>1003027198</v>
+      </c>
+      <c r="G26" s="45">
+        <v>5</v>
+      </c>
+      <c r="H26" s="45">
+        <v>5</v>
+      </c>
+      <c r="I26" s="45">
+        <v>4</v>
+      </c>
+      <c r="J26" s="45">
+        <v>4</v>
+      </c>
+      <c r="K26" s="45">
+        <v>4</v>
+      </c>
+      <c r="L26" s="45">
+        <v>4</v>
+      </c>
+      <c r="M26" s="45">
+        <v>5</v>
+      </c>
+      <c r="N26" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G26:M26),"-")</f>
+        <v>4.4285714285714288</v>
+      </c>
+      <c r="O26" s="46" t="str" cm="1">
+        <f t="array" ref="O26">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A27" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B27" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C27" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D27" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E27" s="43" t="s">
+        <v>64</v>
+      </c>
+      <c r="F27" s="44">
+        <v>1035017030</v>
+      </c>
+      <c r="G27" s="45">
+        <v>5</v>
+      </c>
+      <c r="H27" s="45">
+        <v>5</v>
+      </c>
+      <c r="I27" s="45">
+        <v>5</v>
+      </c>
+      <c r="J27" s="45">
+        <v>3</v>
+      </c>
+      <c r="K27" s="45">
+        <v>4</v>
+      </c>
+      <c r="L27" s="45">
+        <v>3</v>
+      </c>
+      <c r="M27" s="45">
+        <v>5</v>
+      </c>
+      <c r="N27" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G27:M27),"-")</f>
+        <v>4.2857142857142856</v>
+      </c>
+      <c r="O27" s="46" t="str" cm="1">
+        <f t="array" ref="O27">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A28" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B28" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C28" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D28" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E28" s="43" t="s">
+        <v>109</v>
+      </c>
+      <c r="F28" s="44">
+        <v>1062424218</v>
+      </c>
+      <c r="G28" s="45">
+        <v>5</v>
+      </c>
+      <c r="H28" s="45">
+        <v>5</v>
+      </c>
+      <c r="I28" s="45">
+        <v>5</v>
+      </c>
+      <c r="J28" s="45">
+        <v>4</v>
+      </c>
+      <c r="K28" s="45">
+        <v>4</v>
+      </c>
+      <c r="L28" s="45">
+        <v>4</v>
+      </c>
+      <c r="M28" s="45">
+        <v>5</v>
+      </c>
+      <c r="N28" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G28:M28),"-")</f>
+        <v>4.5714285714285712</v>
+      </c>
+      <c r="O28" s="46" t="str" cm="1">
+        <f t="array" ref="O28">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A29" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B29" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C29" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D29" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E29" s="43" t="s">
+        <v>106</v>
+      </c>
+      <c r="F29" s="44">
+        <v>1062436143</v>
+      </c>
+      <c r="G29" s="45">
+        <v>5</v>
+      </c>
+      <c r="H29" s="45">
+        <v>5</v>
+      </c>
+      <c r="I29" s="45">
+        <v>3</v>
+      </c>
+      <c r="J29" s="45">
+        <v>3</v>
+      </c>
+      <c r="K29" s="45">
+        <v>2</v>
+      </c>
+      <c r="L29" s="45">
+        <v>2</v>
+      </c>
+      <c r="M29" s="45">
+        <v>5</v>
+      </c>
+      <c r="N29" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G29:M29),"-")</f>
+        <v>3.5714285714285716</v>
+      </c>
+      <c r="O29" s="46" t="str" cm="1">
+        <f t="array" ref="O29">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A30" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B30" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C30" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D30" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E30" s="43" t="s">
+        <v>100</v>
+      </c>
+      <c r="F30" s="44">
+        <v>1062444411</v>
+      </c>
+      <c r="G30" s="45">
+        <v>5</v>
+      </c>
+      <c r="H30" s="45">
+        <v>5</v>
+      </c>
+      <c r="I30" s="45">
+        <v>5</v>
+      </c>
+      <c r="J30" s="45">
+        <v>5</v>
+      </c>
+      <c r="K30" s="45">
+        <v>5</v>
+      </c>
+      <c r="L30" s="45">
+        <v>5</v>
+      </c>
+      <c r="M30" s="45">
+        <v>5</v>
+      </c>
+      <c r="N30" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G30:M30),"-")</f>
+        <v>5</v>
+      </c>
+      <c r="O30" s="46" t="str" cm="1">
+        <f t="array" ref="O30">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>CAMBIA A NIVEL 2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A31" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B31" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C31" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D31" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E31" s="43" t="s">
+        <v>79</v>
+      </c>
+      <c r="F31" s="44">
+        <v>1062540875</v>
+      </c>
+      <c r="G31" s="45">
+        <v>5</v>
+      </c>
+      <c r="H31" s="45">
+        <v>5</v>
+      </c>
+      <c r="I31" s="45">
+        <v>3</v>
+      </c>
+      <c r="J31" s="45">
+        <v>3</v>
+      </c>
+      <c r="K31" s="45">
+        <v>3</v>
+      </c>
+      <c r="L31" s="45">
+        <v>2</v>
+      </c>
+      <c r="M31" s="45">
+        <v>4</v>
+      </c>
+      <c r="N31" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G31:M31),"-")</f>
+        <v>3.5714285714285716</v>
+      </c>
+      <c r="O31" s="46" t="str" cm="1">
+        <f t="array" ref="O31">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A32" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B32" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C32" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D32" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E32" s="43" t="s">
+        <v>99</v>
+      </c>
+      <c r="F32" s="44">
+        <v>1062544508</v>
+      </c>
+      <c r="G32" s="45">
+        <v>5</v>
+      </c>
+      <c r="H32" s="45">
+        <v>5</v>
+      </c>
+      <c r="I32" s="45">
+        <v>5</v>
+      </c>
+      <c r="J32" s="45">
+        <v>4</v>
+      </c>
+      <c r="K32" s="45">
+        <v>4</v>
+      </c>
+      <c r="L32" s="45">
+        <v>4</v>
+      </c>
+      <c r="M32" s="45">
+        <v>5</v>
+      </c>
+      <c r="N32" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G32:M32),"-")</f>
+        <v>4.5714285714285712</v>
+      </c>
+      <c r="O32" s="46" t="str" cm="1">
+        <f t="array" ref="O32">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A33" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B33" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C33" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D33" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E33" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="F33" s="44">
+        <v>1062546526</v>
+      </c>
+      <c r="G33" s="45">
+        <v>5</v>
+      </c>
+      <c r="H33" s="45">
+        <v>5</v>
+      </c>
+      <c r="I33" s="45">
+        <v>3</v>
+      </c>
+      <c r="J33" s="45">
+        <v>3</v>
+      </c>
+      <c r="K33" s="45">
+        <v>3</v>
+      </c>
+      <c r="L33" s="45">
+        <v>2</v>
+      </c>
+      <c r="M33" s="45">
+        <v>5</v>
+      </c>
+      <c r="N33" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G33:M33),"-")</f>
+        <v>3.7142857142857144</v>
+      </c>
+      <c r="O33" s="46" t="str" cm="1">
+        <f t="array" ref="O33">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A34" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B34" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C34" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D34" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E34" s="43" t="s">
+        <v>68</v>
+      </c>
+      <c r="F34" s="44">
+        <v>1062966144</v>
+      </c>
+      <c r="G34" s="45">
+        <v>5</v>
+      </c>
+      <c r="H34" s="45">
+        <v>5</v>
+      </c>
+      <c r="I34" s="45">
+        <v>5</v>
+      </c>
+      <c r="J34" s="45">
+        <v>4</v>
+      </c>
+      <c r="K34" s="45">
+        <v>4</v>
+      </c>
+      <c r="L34" s="45">
+        <v>4</v>
+      </c>
+      <c r="M34" s="45">
+        <v>5</v>
+      </c>
+      <c r="N34" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G34:M34),"-")</f>
+        <v>4.5714285714285712</v>
+      </c>
+      <c r="O34" s="46" t="str" cm="1">
+        <f t="array" ref="O34">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A35" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B35" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C35" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D35" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E35" s="43" t="s">
+        <v>105</v>
+      </c>
+      <c r="F35" s="44">
+        <v>1067940515</v>
+      </c>
+      <c r="G35" s="45">
+        <v>5</v>
+      </c>
+      <c r="H35" s="45">
+        <v>5</v>
+      </c>
+      <c r="I35" s="45">
+        <v>4</v>
+      </c>
+      <c r="J35" s="45">
+        <v>3</v>
+      </c>
+      <c r="K35" s="45">
+        <v>4</v>
+      </c>
+      <c r="L35" s="45">
+        <v>3</v>
+      </c>
+      <c r="M35" s="45">
+        <v>5</v>
+      </c>
+      <c r="N35" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G35:M35),"-")</f>
+        <v>4.1428571428571432</v>
+      </c>
+      <c r="O35" s="46" t="str" cm="1">
+        <f t="array" ref="O35">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A36" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B36" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C36" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D36" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E36" s="43" t="s">
+        <v>67</v>
+      </c>
+      <c r="F36" s="44">
+        <v>1067945529</v>
+      </c>
+      <c r="G36" s="45">
+        <v>5</v>
+      </c>
+      <c r="H36" s="45">
+        <v>5</v>
+      </c>
+      <c r="I36" s="45">
+        <v>5</v>
+      </c>
+      <c r="J36" s="45">
+        <v>4</v>
+      </c>
+      <c r="K36" s="45">
+        <v>4</v>
+      </c>
+      <c r="L36" s="45">
+        <v>4</v>
+      </c>
+      <c r="M36" s="45">
+        <v>5</v>
+      </c>
+      <c r="N36" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G36:M36),"-")</f>
+        <v>4.5714285714285712</v>
+      </c>
+      <c r="O36" s="46" t="str" cm="1">
+        <f t="array" ref="O36">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A37" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B37" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C37" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D37" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E37" s="43" t="s">
+        <v>71</v>
+      </c>
+      <c r="F37" s="44">
+        <v>1067956606</v>
+      </c>
+      <c r="G37" s="45">
+        <v>5</v>
+      </c>
+      <c r="H37" s="45">
+        <v>5</v>
+      </c>
+      <c r="I37" s="45">
+        <v>5</v>
+      </c>
+      <c r="J37" s="45">
+        <v>5</v>
+      </c>
+      <c r="K37" s="45">
+        <v>5</v>
+      </c>
+      <c r="L37" s="45">
+        <v>5</v>
+      </c>
+      <c r="M37" s="45">
+        <v>5</v>
+      </c>
+      <c r="N37" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G37:M37),"-")</f>
+        <v>5</v>
+      </c>
+      <c r="O37" s="46" t="str" cm="1">
+        <f t="array" ref="O37">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>CAMBIA A NIVEL 2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A38" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B38" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C38" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D38" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E38" s="43" t="s">
+        <v>101</v>
+      </c>
+      <c r="F38" s="44">
+        <v>1068441879</v>
+      </c>
+      <c r="G38" s="45">
+        <v>5</v>
+      </c>
+      <c r="H38" s="45">
+        <v>3</v>
+      </c>
+      <c r="I38" s="45">
+        <v>2</v>
+      </c>
+      <c r="J38" s="45">
+        <v>3</v>
+      </c>
+      <c r="K38" s="45">
+        <v>2</v>
+      </c>
+      <c r="L38" s="45">
+        <v>2</v>
+      </c>
+      <c r="M38" s="45">
+        <v>4</v>
+      </c>
+      <c r="N38" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G38:M38),"-")</f>
+        <v>3</v>
+      </c>
+      <c r="O38" s="46" t="str" cm="1">
+        <f t="array" ref="O38">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A39" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B39" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C39" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D39" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E39" s="43" t="s">
+        <v>104</v>
+      </c>
+      <c r="F39" s="44">
+        <v>1068442748</v>
+      </c>
+      <c r="G39" s="45">
+        <v>5</v>
+      </c>
+      <c r="H39" s="45">
+        <v>1</v>
+      </c>
+      <c r="I39" s="45">
+        <v>2</v>
+      </c>
+      <c r="J39" s="45">
+        <v>1</v>
+      </c>
+      <c r="K39" s="45">
+        <v>1</v>
+      </c>
+      <c r="L39" s="45">
+        <v>1</v>
+      </c>
+      <c r="M39" s="45">
+        <v>1</v>
+      </c>
+      <c r="N39" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G39:M39),"-")</f>
+        <v>1.7142857142857142</v>
+      </c>
+      <c r="O39" s="46" t="str" cm="1">
+        <f t="array" ref="O39">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A40" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B40" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C40" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D40" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E40" s="43" t="s">
+        <v>77</v>
+      </c>
+      <c r="F40" s="44">
+        <v>1068443767</v>
+      </c>
+      <c r="G40" s="45">
+        <v>5</v>
+      </c>
+      <c r="H40" s="45">
+        <v>3</v>
+      </c>
+      <c r="I40" s="45">
+        <v>2</v>
+      </c>
+      <c r="J40" s="45">
+        <v>2</v>
+      </c>
+      <c r="K40" s="45">
+        <v>2</v>
+      </c>
+      <c r="L40" s="45">
+        <v>2</v>
+      </c>
+      <c r="M40" s="45">
+        <v>5</v>
+      </c>
+      <c r="N40" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G40:M40),"-")</f>
+        <v>3</v>
+      </c>
+      <c r="O40" s="46" t="str" cm="1">
+        <f t="array" ref="O40">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A41" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B41" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C41" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D41" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E41" s="43" t="s">
+        <v>63</v>
+      </c>
+      <c r="F41" s="44">
+        <v>1073824962</v>
+      </c>
+      <c r="G41" s="45">
+        <v>5</v>
+      </c>
+      <c r="H41" s="45">
+        <v>5</v>
+      </c>
+      <c r="I41" s="45">
+        <v>5</v>
+      </c>
+      <c r="J41" s="45">
+        <v>4</v>
+      </c>
+      <c r="K41" s="45">
+        <v>5</v>
+      </c>
+      <c r="L41" s="45">
+        <v>4</v>
+      </c>
+      <c r="M41" s="45">
+        <v>5</v>
+      </c>
+      <c r="N41" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G41:M41),"-")</f>
+        <v>4.7142857142857144</v>
+      </c>
+      <c r="O41" s="46" t="str" cm="1">
+        <f t="array" ref="O41">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>CAMBIA A NIVEL 2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A42" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B42" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C42" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D42" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E42" s="43" t="s">
+        <v>76</v>
+      </c>
+      <c r="F42" s="44">
+        <v>1126253349</v>
+      </c>
+      <c r="G42" s="45">
+        <v>5</v>
+      </c>
+      <c r="H42" s="45">
+        <v>5</v>
+      </c>
+      <c r="I42" s="45">
+        <v>4</v>
+      </c>
+      <c r="J42" s="45">
+        <v>4</v>
+      </c>
+      <c r="K42" s="45">
+        <v>4</v>
+      </c>
+      <c r="L42" s="45">
+        <v>5</v>
+      </c>
+      <c r="M42" s="45">
+        <v>5</v>
+      </c>
+      <c r="N42" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G42:M42),"-")</f>
+        <v>4.5714285714285712</v>
+      </c>
+      <c r="O42" s="46" t="str" cm="1">
+        <f t="array" ref="O42">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A43" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B43" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C43" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D43" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E43" s="43" t="s">
+        <v>103</v>
+      </c>
+      <c r="F43" s="44">
+        <v>1137975856</v>
+      </c>
+      <c r="G43" s="45">
+        <v>5</v>
+      </c>
+      <c r="H43" s="45">
+        <v>5</v>
+      </c>
+      <c r="I43" s="45">
+        <v>5</v>
+      </c>
+      <c r="J43" s="45">
+        <v>4</v>
+      </c>
+      <c r="K43" s="45">
+        <v>4</v>
+      </c>
+      <c r="L43" s="45">
+        <v>4</v>
+      </c>
+      <c r="M43" s="45">
+        <v>5</v>
+      </c>
+      <c r="N43" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G43:M43),"-")</f>
+        <v>4.5714285714285712</v>
+      </c>
+      <c r="O43" s="46" t="str" cm="1">
+        <f t="array" ref="O43">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A44" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B44" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C44" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D44" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E44" s="43" t="s">
+        <v>102</v>
+      </c>
+      <c r="F44" s="44">
+        <v>1138030749</v>
+      </c>
+      <c r="G44" s="45">
+        <v>5</v>
+      </c>
+      <c r="H44" s="45">
+        <v>5</v>
+      </c>
+      <c r="I44" s="45">
+        <v>4</v>
+      </c>
+      <c r="J44" s="45">
+        <v>4</v>
+      </c>
+      <c r="K44" s="45">
+        <v>4</v>
+      </c>
+      <c r="L44" s="45">
+        <v>4</v>
+      </c>
+      <c r="M44" s="45">
+        <v>5</v>
+      </c>
+      <c r="N44" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G44:M44),"-")</f>
+        <v>4.4285714285714288</v>
+      </c>
+      <c r="O44" s="46" t="str" cm="1">
+        <f t="array" ref="O44">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A45" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B45" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C45" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D45" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E45" s="43" t="s">
+        <v>107</v>
+      </c>
+      <c r="F45" s="44">
+        <v>1138031920</v>
+      </c>
+      <c r="G45" s="45">
+        <v>5</v>
+      </c>
+      <c r="H45" s="45">
+        <v>5</v>
+      </c>
+      <c r="I45" s="45">
+        <v>5</v>
+      </c>
+      <c r="J45" s="45">
+        <v>4</v>
+      </c>
+      <c r="K45" s="45">
+        <v>5</v>
+      </c>
+      <c r="L45" s="45">
+        <v>4</v>
+      </c>
+      <c r="M45" s="45">
+        <v>5</v>
+      </c>
+      <c r="N45" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G45:M45),"-")</f>
+        <v>4.7142857142857144</v>
+      </c>
+      <c r="O45" s="46" t="str" cm="1">
+        <f t="array" ref="O45">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>CAMBIA A NIVEL 2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A46" s="40">
+        <f>MONTH(NIVEL_1[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B46" s="41" t="str">
+        <f>IF(NIVEL_1[[#This Row],['#]]&gt;0,"NIVEL 1","")</f>
+        <v>NIVEL 1</v>
+      </c>
+      <c r="C46" s="41" t="str">
+        <f>TEXT(NIVEL_1[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D46" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E46" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="F46" s="44">
+        <v>1233348383</v>
+      </c>
+      <c r="G46" s="45">
+        <v>5</v>
+      </c>
+      <c r="H46" s="45">
+        <v>2</v>
+      </c>
+      <c r="I46" s="45">
+        <v>2</v>
+      </c>
+      <c r="J46" s="45">
+        <v>2</v>
+      </c>
+      <c r="K46" s="45">
+        <v>2</v>
+      </c>
+      <c r="L46" s="45">
+        <v>2</v>
+      </c>
+      <c r="M46" s="45">
+        <v>4</v>
+      </c>
+      <c r="N46" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 1'!G46:M46),"-")</f>
+        <v>2.7142857142857144</v>
+      </c>
+      <c r="O46" s="46" t="str" cm="1">
+        <f t="array" ref="O46">_xlfn.IFS(NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 2",NIVEL_1[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
         <v>-</v>
       </c>
     </row>
@@ -14170,7 +15358,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.44140625" customWidth="1"/>
@@ -14725,6 +15913,630 @@
         <v>-</v>
       </c>
     </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A12" s="45">
+        <f>MONTH(NIVEL_2[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B12" s="47" t="str">
+        <f>IF(NIVEL_2[[#This Row],['#]]&gt;0,"NIVEL 2","")</f>
+        <v>NIVEL 2</v>
+      </c>
+      <c r="C12" s="47" t="str">
+        <f>TEXT(NIVEL_2[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D12" s="42">
+        <v>46110</v>
+      </c>
+      <c r="E12" s="43" t="s">
+        <v>82</v>
+      </c>
+      <c r="F12" s="45">
+        <v>1027663882</v>
+      </c>
+      <c r="G12" s="45">
+        <v>4</v>
+      </c>
+      <c r="H12" s="45">
+        <v>4</v>
+      </c>
+      <c r="I12" s="45">
+        <v>4</v>
+      </c>
+      <c r="J12" s="45">
+        <v>4</v>
+      </c>
+      <c r="K12" s="45">
+        <v>3</v>
+      </c>
+      <c r="L12" s="45">
+        <v>5</v>
+      </c>
+      <c r="M12" s="45">
+        <v>3</v>
+      </c>
+      <c r="N12" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 2'!G12:M12),"-")</f>
+        <v>3.8571428571428572</v>
+      </c>
+      <c r="O12" s="48" t="str" cm="1">
+        <f t="array" ref="O12">_xlfn.IFS(NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 3",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A13" s="45">
+        <f>MONTH(NIVEL_2[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B13" s="47" t="str">
+        <f>IF(NIVEL_2[[#This Row],['#]]&gt;0,"NIVEL 2","")</f>
+        <v>NIVEL 2</v>
+      </c>
+      <c r="C13" s="47" t="str">
+        <f>TEXT(NIVEL_2[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D13" s="42">
+        <v>46110</v>
+      </c>
+      <c r="E13" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="F13" s="45">
+        <v>1035003918</v>
+      </c>
+      <c r="G13" s="45">
+        <v>5</v>
+      </c>
+      <c r="H13" s="45">
+        <v>4</v>
+      </c>
+      <c r="I13" s="45">
+        <v>4</v>
+      </c>
+      <c r="J13" s="45">
+        <v>4</v>
+      </c>
+      <c r="K13" s="45">
+        <v>4</v>
+      </c>
+      <c r="L13" s="45">
+        <v>5</v>
+      </c>
+      <c r="M13" s="45">
+        <v>2</v>
+      </c>
+      <c r="N13" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 2'!G13:M13),"-")</f>
+        <v>4</v>
+      </c>
+      <c r="O13" s="48" t="str" cm="1">
+        <f t="array" ref="O13">_xlfn.IFS(NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 3",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A14" s="45">
+        <f>MONTH(NIVEL_2[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B14" s="47" t="str">
+        <f>IF(NIVEL_2[[#This Row],['#]]&gt;0,"NIVEL 2","")</f>
+        <v>NIVEL 2</v>
+      </c>
+      <c r="C14" s="47" t="str">
+        <f>TEXT(NIVEL_2[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D14" s="42">
+        <v>46110</v>
+      </c>
+      <c r="E14" s="43" t="s">
+        <v>111</v>
+      </c>
+      <c r="F14" s="45">
+        <v>1062980565</v>
+      </c>
+      <c r="G14" s="45">
+        <v>4</v>
+      </c>
+      <c r="H14" s="45">
+        <v>4</v>
+      </c>
+      <c r="I14" s="45">
+        <v>2</v>
+      </c>
+      <c r="J14" s="45">
+        <v>3</v>
+      </c>
+      <c r="K14" s="45">
+        <v>3</v>
+      </c>
+      <c r="L14" s="45">
+        <v>5</v>
+      </c>
+      <c r="M14" s="45">
+        <v>2</v>
+      </c>
+      <c r="N14" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 2'!G14:M14),"-")</f>
+        <v>3.2857142857142856</v>
+      </c>
+      <c r="O14" s="48" t="str" cm="1">
+        <f t="array" ref="O14">_xlfn.IFS(NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 3",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15" s="45">
+        <f>MONTH(NIVEL_2[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B15" s="47" t="str">
+        <f>IF(NIVEL_2[[#This Row],['#]]&gt;0,"NIVEL 2","")</f>
+        <v>NIVEL 2</v>
+      </c>
+      <c r="C15" s="47" t="str">
+        <f>TEXT(NIVEL_2[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D15" s="42">
+        <v>46110</v>
+      </c>
+      <c r="E15" s="43" t="s">
+        <v>81</v>
+      </c>
+      <c r="F15" s="45">
+        <v>1062981643</v>
+      </c>
+      <c r="G15" s="45">
+        <v>4</v>
+      </c>
+      <c r="H15" s="45">
+        <v>5</v>
+      </c>
+      <c r="I15" s="45">
+        <v>2</v>
+      </c>
+      <c r="J15" s="45">
+        <v>3</v>
+      </c>
+      <c r="K15" s="45">
+        <v>3</v>
+      </c>
+      <c r="L15" s="45">
+        <v>4</v>
+      </c>
+      <c r="M15" s="45">
+        <v>2</v>
+      </c>
+      <c r="N15" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 2'!G15:M15),"-")</f>
+        <v>3.2857142857142856</v>
+      </c>
+      <c r="O15" s="48" t="str" cm="1">
+        <f t="array" ref="O15">_xlfn.IFS(NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 3",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A16" s="45">
+        <f>MONTH(NIVEL_2[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B16" s="47" t="str">
+        <f>IF(NIVEL_2[[#This Row],['#]]&gt;0,"NIVEL 2","")</f>
+        <v>NIVEL 2</v>
+      </c>
+      <c r="C16" s="47" t="str">
+        <f>TEXT(NIVEL_2[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D16" s="42">
+        <v>46110</v>
+      </c>
+      <c r="E16" s="43" t="s">
+        <v>112</v>
+      </c>
+      <c r="F16" s="45">
+        <v>1066747786</v>
+      </c>
+      <c r="G16" s="45">
+        <v>5</v>
+      </c>
+      <c r="H16" s="45">
+        <v>4</v>
+      </c>
+      <c r="I16" s="45">
+        <v>4</v>
+      </c>
+      <c r="J16" s="45">
+        <v>4</v>
+      </c>
+      <c r="K16" s="45">
+        <v>4</v>
+      </c>
+      <c r="L16" s="45">
+        <v>5</v>
+      </c>
+      <c r="M16" s="45">
+        <v>2</v>
+      </c>
+      <c r="N16" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 2'!G16:M16),"-")</f>
+        <v>4</v>
+      </c>
+      <c r="O16" s="48" t="str" cm="1">
+        <f t="array" ref="O16">_xlfn.IFS(NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 3",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A17" s="45">
+        <f>MONTH(NIVEL_2[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B17" s="47" t="str">
+        <f>IF(NIVEL_2[[#This Row],['#]]&gt;0,"NIVEL 2","")</f>
+        <v>NIVEL 2</v>
+      </c>
+      <c r="C17" s="47" t="str">
+        <f>TEXT(NIVEL_2[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D17" s="42">
+        <v>46111</v>
+      </c>
+      <c r="E17" s="43" t="s">
+        <v>65</v>
+      </c>
+      <c r="F17" s="45">
+        <v>1067859838</v>
+      </c>
+      <c r="G17" s="45">
+        <v>4</v>
+      </c>
+      <c r="H17" s="45">
+        <v>4</v>
+      </c>
+      <c r="I17" s="45">
+        <v>2</v>
+      </c>
+      <c r="J17" s="45">
+        <v>4</v>
+      </c>
+      <c r="K17" s="45">
+        <v>4</v>
+      </c>
+      <c r="L17" s="45">
+        <v>5</v>
+      </c>
+      <c r="M17" s="45">
+        <v>1</v>
+      </c>
+      <c r="N17" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 2'!G17:M17),"-")</f>
+        <v>3.4285714285714284</v>
+      </c>
+      <c r="O17" s="48" t="str" cm="1">
+        <f t="array" ref="O17">_xlfn.IFS(NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 3",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A18" s="45">
+        <f>MONTH(NIVEL_2[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B18" s="47" t="str">
+        <f>IF(NIVEL_2[[#This Row],['#]]&gt;0,"NIVEL 2","")</f>
+        <v>NIVEL 2</v>
+      </c>
+      <c r="C18" s="47" t="str">
+        <f>TEXT(NIVEL_2[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D18" s="42">
+        <v>46110</v>
+      </c>
+      <c r="E18" s="43" t="s">
+        <v>113</v>
+      </c>
+      <c r="F18" s="45">
+        <v>1068439668</v>
+      </c>
+      <c r="G18" s="45">
+        <v>5</v>
+      </c>
+      <c r="H18" s="45">
+        <v>5</v>
+      </c>
+      <c r="I18" s="45">
+        <v>4</v>
+      </c>
+      <c r="J18" s="45">
+        <v>4</v>
+      </c>
+      <c r="K18" s="45">
+        <v>3</v>
+      </c>
+      <c r="L18" s="45">
+        <v>5</v>
+      </c>
+      <c r="M18" s="45">
+        <v>3</v>
+      </c>
+      <c r="N18" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 2'!G18:M18),"-")</f>
+        <v>4.1428571428571432</v>
+      </c>
+      <c r="O18" s="48" t="str" cm="1">
+        <f t="array" ref="O18">_xlfn.IFS(NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 3",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A19" s="45">
+        <f>MONTH(NIVEL_2[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B19" s="47" t="str">
+        <f>IF(NIVEL_2[[#This Row],['#]]&gt;0,"NIVEL 2","")</f>
+        <v>NIVEL 2</v>
+      </c>
+      <c r="C19" s="47" t="str">
+        <f>TEXT(NIVEL_2[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D19" s="42">
+        <v>46110</v>
+      </c>
+      <c r="E19" s="43" t="s">
+        <v>72</v>
+      </c>
+      <c r="F19" s="45">
+        <v>1073817245</v>
+      </c>
+      <c r="G19" s="45">
+        <v>5</v>
+      </c>
+      <c r="H19" s="45">
+        <v>4</v>
+      </c>
+      <c r="I19" s="45">
+        <v>2</v>
+      </c>
+      <c r="J19" s="45">
+        <v>3</v>
+      </c>
+      <c r="K19" s="45">
+        <v>2</v>
+      </c>
+      <c r="L19" s="45">
+        <v>5</v>
+      </c>
+      <c r="M19" s="45">
+        <v>2</v>
+      </c>
+      <c r="N19" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 2'!G19:M19),"-")</f>
+        <v>3.2857142857142856</v>
+      </c>
+      <c r="O19" s="48" t="str" cm="1">
+        <f t="array" ref="O19">_xlfn.IFS(NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 3",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A20" s="45">
+        <f>MONTH(NIVEL_2[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B20" s="47" t="str">
+        <f>IF(NIVEL_2[[#This Row],['#]]&gt;0,"NIVEL 2","")</f>
+        <v>NIVEL 2</v>
+      </c>
+      <c r="C20" s="47" t="str">
+        <f>TEXT(NIVEL_2[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D20" s="42">
+        <v>46110</v>
+      </c>
+      <c r="E20" s="43" t="s">
+        <v>84</v>
+      </c>
+      <c r="F20" s="45">
+        <v>1104267144</v>
+      </c>
+      <c r="G20" s="45">
+        <v>4</v>
+      </c>
+      <c r="H20" s="45">
+        <v>4</v>
+      </c>
+      <c r="I20" s="45">
+        <v>3</v>
+      </c>
+      <c r="J20" s="45">
+        <v>3</v>
+      </c>
+      <c r="K20" s="45">
+        <v>5</v>
+      </c>
+      <c r="L20" s="45">
+        <v>4</v>
+      </c>
+      <c r="M20" s="45">
+        <v>3</v>
+      </c>
+      <c r="N20" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 2'!G20:M20),"-")</f>
+        <v>3.7142857142857144</v>
+      </c>
+      <c r="O20" s="48" t="str" cm="1">
+        <f t="array" ref="O20">_xlfn.IFS(NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 3",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A21" s="45">
+        <f>MONTH(NIVEL_2[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B21" s="47" t="str">
+        <f>IF(NIVEL_2[[#This Row],['#]]&gt;0,"NIVEL 2","")</f>
+        <v>NIVEL 2</v>
+      </c>
+      <c r="C21" s="47" t="str">
+        <f>TEXT(NIVEL_2[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D21" s="42">
+        <v>46110</v>
+      </c>
+      <c r="E21" s="43" t="s">
+        <v>114</v>
+      </c>
+      <c r="F21" s="45">
+        <v>1138031207</v>
+      </c>
+      <c r="G21" s="45">
+        <v>5</v>
+      </c>
+      <c r="H21" s="45">
+        <v>4</v>
+      </c>
+      <c r="I21" s="45">
+        <v>3</v>
+      </c>
+      <c r="J21" s="45">
+        <v>3</v>
+      </c>
+      <c r="K21" s="45">
+        <v>3</v>
+      </c>
+      <c r="L21" s="45">
+        <v>5</v>
+      </c>
+      <c r="M21" s="45">
+        <v>3</v>
+      </c>
+      <c r="N21" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 2'!G21:M21),"-")</f>
+        <v>3.7142857142857144</v>
+      </c>
+      <c r="O21" s="48" t="str" cm="1">
+        <f t="array" ref="O21">_xlfn.IFS(NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 3",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A22" s="45">
+        <f>MONTH(NIVEL_2[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B22" s="47" t="str">
+        <f>IF(NIVEL_2[[#This Row],['#]]&gt;0,"NIVEL 2","")</f>
+        <v>NIVEL 2</v>
+      </c>
+      <c r="C22" s="47" t="str">
+        <f>TEXT(NIVEL_2[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D22" s="42">
+        <v>46110</v>
+      </c>
+      <c r="E22" s="43" t="s">
+        <v>83</v>
+      </c>
+      <c r="F22" s="45">
+        <v>1138032549</v>
+      </c>
+      <c r="G22" s="45">
+        <v>4</v>
+      </c>
+      <c r="H22" s="45">
+        <v>5</v>
+      </c>
+      <c r="I22" s="45">
+        <v>3</v>
+      </c>
+      <c r="J22" s="45">
+        <v>3</v>
+      </c>
+      <c r="K22" s="45">
+        <v>5</v>
+      </c>
+      <c r="L22" s="45">
+        <v>5</v>
+      </c>
+      <c r="M22" s="45">
+        <v>5</v>
+      </c>
+      <c r="N22" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 2'!G22:M22),"-")</f>
+        <v>4.2857142857142856</v>
+      </c>
+      <c r="O22" s="48" t="str" cm="1">
+        <f t="array" ref="O22">_xlfn.IFS(NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 3",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A23" s="45">
+        <f>MONTH(NIVEL_2[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B23" s="47" t="str">
+        <f>IF(NIVEL_2[[#This Row],['#]]&gt;0,"NIVEL 2","")</f>
+        <v>NIVEL 2</v>
+      </c>
+      <c r="C23" s="47" t="str">
+        <f>TEXT(NIVEL_2[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D23" s="42">
+        <v>46110</v>
+      </c>
+      <c r="E23" s="43" t="s">
+        <v>73</v>
+      </c>
+      <c r="F23" s="45">
+        <v>1140444971</v>
+      </c>
+      <c r="G23" s="45">
+        <v>5</v>
+      </c>
+      <c r="H23" s="45">
+        <v>4</v>
+      </c>
+      <c r="I23" s="45">
+        <v>4</v>
+      </c>
+      <c r="J23" s="45">
+        <v>4</v>
+      </c>
+      <c r="K23" s="45">
+        <v>3</v>
+      </c>
+      <c r="L23" s="45">
+        <v>5</v>
+      </c>
+      <c r="M23" s="45">
+        <v>3</v>
+      </c>
+      <c r="N23" s="19">
+        <f>IFERROR(AVERAGE('NIVEL 2'!G23:M23),"-")</f>
+        <v>4</v>
+      </c>
+      <c r="O23" s="48" t="str" cm="1">
+        <f t="array" ref="O23">_xlfn.IFS(NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]="-","-",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&gt;=4.7,"CAMBIA A NIVEL 3",NIVEL_2[[#This Row],[Pase de Nivel 4,7 ptos]]&lt;=4.7,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
@@ -14749,7 +16561,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.33203125" customWidth="1"/>
@@ -15067,6 +16879,76 @@
       </c>
       <c r="U5" s="32" t="str" cm="1">
         <f t="array" ref="U5">_xlfn.IFS(NIVEL_3[[#This Row],[Pase de Nivel 4,9 ptos]]="-","-",NIVEL_3[[#This Row],[Pase de Nivel 4,9 ptos]]&gt;=4.9,"CAMBIA A EQUIPO",NIVEL_3[[#This Row],[Pase de Nivel 4,9 ptos]]&lt;=4.9,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A6" s="49">
+        <f>MONTH(NIVEL_3[[#This Row],[Fecha de Evaluación]])</f>
+        <v>3</v>
+      </c>
+      <c r="B6" s="41" t="str">
+        <f>IF(NIVEL_3[[#This Row],['#]]&gt;0,"NIVEL 3","")</f>
+        <v>NIVEL 3</v>
+      </c>
+      <c r="C6" s="50" t="str">
+        <f>TEXT(NIVEL_3[[#This Row],[Fecha de Evaluación]],"MMMM")</f>
+        <v>marzo</v>
+      </c>
+      <c r="D6" s="51">
+        <v>46110</v>
+      </c>
+      <c r="E6" s="52" t="s">
+        <v>85</v>
+      </c>
+      <c r="F6" s="53">
+        <v>1062539643</v>
+      </c>
+      <c r="G6" s="53">
+        <v>4</v>
+      </c>
+      <c r="H6" s="53">
+        <v>4</v>
+      </c>
+      <c r="I6" s="53">
+        <v>5</v>
+      </c>
+      <c r="J6" s="53">
+        <v>5</v>
+      </c>
+      <c r="K6" s="53">
+        <v>4</v>
+      </c>
+      <c r="L6" s="53">
+        <v>3</v>
+      </c>
+      <c r="M6" s="53">
+        <v>5</v>
+      </c>
+      <c r="N6" s="53">
+        <v>4</v>
+      </c>
+      <c r="O6" s="53">
+        <v>4</v>
+      </c>
+      <c r="P6" s="53">
+        <v>5</v>
+      </c>
+      <c r="Q6" s="53">
+        <v>3</v>
+      </c>
+      <c r="R6" s="53">
+        <v>3</v>
+      </c>
+      <c r="S6" s="53">
+        <v>4</v>
+      </c>
+      <c r="T6" s="54">
+        <f>IFERROR(AVERAGE(G6:S6),"-")</f>
+        <v>4.0769230769230766</v>
+      </c>
+      <c r="U6" s="55" t="str" cm="1">
+        <f t="array" ref="U6">_xlfn.IFS(NIVEL_3[[#This Row],[Pase de Nivel 4,9 ptos]]="-","-",NIVEL_3[[#This Row],[Pase de Nivel 4,9 ptos]]&gt;=4.9,"CAMBIA A EQUIPO",NIVEL_3[[#This Row],[Pase de Nivel 4,9 ptos]]&lt;=4.9,"-")</f>
         <v>-</v>
       </c>
     </row>

</xml_diff>